<commit_message>
docs(testing): copy the test-case workbook forward to CAA 251026
The main merge had regenerated yesterday's CAA 241026 in place. Restore it
to main's copy and export today's workbook instead; source-of-truth points
at the new file.

Refs SCRUM-207, E09-S01

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 241026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 241026.xlsx
@@ -15007,25 +15007,25 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>Event "Community Meetup" is open for registration; attendee_e@example.com's account has no contact number. Registration details are the account's name, email address and contact number, so nothing extra is entered at registration (T-32, O-05); every account has an email, so the contact number is the detail that can be missing.</t>
+          <t>Event "Community Meetup" is open for registration</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
           <t>1. Log in as attendee_e@example.com
   2. Open event "Community Meetup"
-  3. Open registration, select a Session and review the details shown from the account
+  3. Leave the Email field empty
   4. Submit registration</t>
         </is>
       </c>
       <c r="I278" s="2" t="inlineStr">
         <is>
-          <t>Name: from account | Email: from account | Contact number: (blank on the account)</t>
+          <t>Name: filled | Email: (blank)</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr">
         <is>
-          <t>Registration is blocked, and Contact number is identified as missing, with a link to add it on the Profile page; no registration is created</t>
+          <t>Registration is blocked, and the Email field is identified as missing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(testing): address PR 332 review comments on booking fixtures
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 241026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 241026.xlsx
@@ -3150,7 +3150,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>E02-S05 - Scenario 1 (Previous event copied; T-99)</t>
+          <t>E02-S05 - Scenario 1 (Previous event copied; assumes O-51)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -8486,7 +8486,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Venue "Riverside Hall" has Setup time 0 and Turnaround time 0 before either booking is created; Confirmed bookings exist for "Charity Run" 15/01/2027 10:00-12:00 (coordinator_1) and "Alumni Dinner" 15/01/2027 12:30-14:00 (coordinator_2); venue_staff_1@connectsphere.com is signed in</t>
+          <t>Venue "Riverside Hall" has Turnaround time 0; Confirmed bookings exist for "Charity Run" 15/01/2027 10:00-12:00 (coordinator_1) and "Alumni Dinner" 15/01/2027 12:30-14:00 (coordinator_2); venue_staff_1@connectsphere.com is signed in</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -10490,7 +10490,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>Venue "Riverside Hall" initially has Setup time 0 and Turnaround time 0 when both bookings are created: "Charity Run" is Confirmed 15/01/2027 10:00-12:00 and "Alumni Dinner" is Pending 15/01/2027 12:30-14:00. Then Setup time is set to 30 and Turnaround time to 45, retaining both bookings; venue_staff_1@connectsphere.com is signed in</t>
+          <t>Venue "Riverside Hall" has Setup time 30 and Turnaround time 45; "Charity Run" is Confirmed 15/01/2027 10:00-12:00; a Pending request for "Alumni Dinner" 15/01/2027 12:30-14:00 was created before the buffers were set; venue_staff_1@connectsphere.com is signed in</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -11048,7 +11048,7 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
+          <t>E06-S06 - Scenario 1 (Overlapping approval blocked)</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -11063,28 +11063,29 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>Verify approval rechecks a confirmed booking after buffer growth</t>
+          <t>Verify that attempting to approve a request that overlaps an existing confirmed booking for the same venue should be blocked with the conflicting booking identified</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>Venue Orchid Hall has setup and turnaround set to 0. Confirmed booking Charity Run occupies 09:00-11:00 and Pending request Product Expo occupies 11:00-13:00; both were accepted while their advertised periods were adjacent. Venue Staff then changes setup time to 30 minutes.</t>
+          <t>"Riverside Hall" has a confirmed booking for "Charity Run" on 15/01/2027, 09:00-17:00. A second pending request for "Riverside Hall" on 15/01/2027, 14:00-18:00 exists for event "Product Expo 2026"</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm the buffer edit saves and both bookings remain present; Pending Product Expo has `buffer_conflict` true while Confirmed Charity Run remains unflagged.
-2. Open Product Expo's Pending request and attempt approval.</t>
+          <t>1. Log in as venue_staff_1@connectsphere.com
+  2. Open the pending request for "Product Expo 2026"
+  3. Attempt to click "Approve"</t>
         </is>
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>Before edit: Charity Run 09:00-11:00; Product Expo 11:00-13:00; both buffers 0. After edit: setup 30 minutes creates a 10:30-11:00 overlap between their buffered windows.</t>
+          <t>Existing confirmed booking: Charity Run, 15/01/2027 09:00-17:00 | Conflicting request: Product Expo 2026, 15/01/2027 14:00-18:00</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>Approval of Product Expo is refused after checking current buffers. Confirmed Charity Run and Pending Product Expo are both retained; Charity Run remains unflagged and Product Expo carries `buffer_conflict` true.</t>
+          <t>Approval is blocked, and the message identifies the existing confirmed "Charity Run" booking as the conflict</t>
         </is>
       </c>
     </row>
@@ -11099,7 +11100,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 2 (Later overlapping claim refused; T-100)</t>
+          <t>E06-S06 - Scenario 2 (Competing request flagged)</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -11114,28 +11115,29 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>Verify a later overlapping request is refused while the first claim remains active</t>
+          <t>Verify that approving one of two pending requests for the same venue and overlapping times should flag the other as conflicting</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>Orchid Hall has no active booking. The setup and turnaround buffers are 30 and 45 minutes. A successfully accepted Pending request for Charity Run occupies advertised time 09:00-11:00.</t>
+          <t>Two pending requests exist for "Riverside Hall" on 20/01/2027, both 09:00-12:00: Request A ("Tech Conference 2026") and Request B ("Product Expo 2026")</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>1. Submit a normal booking request for Product Expo at 10:00-12:00 on Orchid Hall.
-2. Read the original request and the venue's booking list.</t>
+          <t>1. Log in as venue_staff_1@connectsphere.com
+  2. Approve Request A ("Tech Conference 2026")
+  3. Open Request B ("Product Expo 2026")</t>
         </is>
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>First accepted claim: Charity Run, 09:00-11:00. Later overlapping request: Product Expo, 10:00-12:00, same venue.</t>
+          <t>Request A: Tech Conference 2026 (approved) | Request B: Product Expo 2026 (same venue, overlapping time)</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>The second request is refused while Charity Run's claim is active. Charity Run remains unchanged and no overlapping Pending row is created.</t>
+          <t>Request B is now flagged as conflicting and cannot be approved until the conflict is resolved</t>
         </is>
       </c>
     </row>
@@ -11150,12 +11152,12 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 3 (Concurrent claims fail safely; T-100)</t>
+          <t>E06-S06 - Scenario 3 (Simultaneous approval fails safely)</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>3 - Integration / regression</t>
+          <t>4 - Negative</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
@@ -11165,28 +11167,28 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>Verify concurrent overlapping new claims accept only one request</t>
+          <t>Verify that if another Venue Staff member approves a conflicting request moments earlier, a simultaneous approval attempt should fail safely and inform the user the venue has just been taken</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>Orchid Hall has no active booking and has 30-minute setup and 45-minute turnaround buffers. Two assigned Coordinators for separate Approved events submit overlapping booking requests concurrently.</t>
+          <t>Two pending requests exist for "Riverside Hall" on 25/01/2027, overlapping times. venue_staff_2@connectsphere.com approves one of them a moment before venue_staff_1@connectsphere.com processes the other</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
-          <t>1. Submit both requests in parallel transactions for the same venue.
-2. Read both responses, booking rows, event statuses, notifications and audit effects.</t>
+          <t>1. As venue_staff_2@connectsphere.com, approve Request A for "Riverside Hall" on 25/01/2027
+  2. Immediately as venue_staff_1@connectsphere.com, attempt to approve the conflicting Request B for the same venue and overlapping time</t>
         </is>
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>Request A: Charity Run, 09:00-11:00. Request B: Product Expo, 10:00-12:00. Both target Orchid Hall.</t>
+          <t>Request A approved by venue_staff_2@connectsphere.com just before venue_staff_1@connectsphere.com's attempt on Request B</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>Exactly one request is accepted. The loser receives 409; it creates no booking row, event-status change, notification or audit effect. Only the accepted request's effects remain.</t>
+          <t>venue_staff_1@connectsphere.com's approval attempt fails safely, with a message stating the venue has just been taken by another approval</t>
         </is>
       </c>
     </row>
@@ -11201,7 +11203,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
+          <t>E06-S06 · Scenario 1 (Overlapping approval blocked)</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -11216,28 +11218,29 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>Verify exact half-open buffered adjacency is allowed with zero buffers</t>
+          <t>Verify that a booking beginning exactly when another ends is not treated as a conflict</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>Venue Orchid Hall has Setup time 0 and Turnaround time 0 before either booking is created. It has a confirmed booking for 2026-11-10 09:00:00 to 2026-11-10 11:00:00. A pending request exists for the same venue for 2026-11-10 11:00:00 to 2026-11-10 13:00:00</t>
+          <t>Venue Orchid Hall has a confirmed booking for 2026-11-10 09:00:00 to 2026-11-10 11:00:00. A pending request exists for the same venue for 2026-11-10 11:00:00 to 2026-11-10 13:00:00</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>1. Open the Pending Product Expo request.
-2. Approve it and read both bookings on the venue calendar.</t>
+          <t>1. Sign in as Venue Staff
+ 2. Open the pending request for 11:00–13:00
+ 3. Approve it</t>
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>Existing: 09:00-11:00. Requested: 11:00-13:00. Both buffers: 0. Shared half-open boundary: 11:00.</t>
+          <t>Existing: 09:00–11:00 · Requested: 11:00–13:00 · Shared boundary: 11:00</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>Approval succeeds and both bookings are Confirmed. The exact half-open boundary is adjacent, not overlapping.</t>
+          <t>The approval succeeds and both bookings show as Confirmed on the venue calendar. Ranges are half-open, so touching at the boundary is not an overlap</t>
         </is>
       </c>
     </row>
@@ -11252,7 +11255,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
+          <t>E06-S06 · Scenario 1 (Overlapping approval blocked)</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
@@ -11267,28 +11270,29 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>Verify a one-minute overlap is refused before an impossible fixture is inserted</t>
+          <t>Verify that a booking overlapping an existing one by a single minute is blocked</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>Orchid Hall has setup and turnaround set to 0 and one active Confirmed booking for Charity Run from 09:00 to 11:00. No Pending request exists for a conflicting period.</t>
+          <t>Venue Orchid Hall has a confirmed booking for 2026-11-10 09:00:00 to 2026-11-10 11:00:00. A pending request exists for the same venue for 2026-11-10 10:59:00 to 2026-11-10 13:00:00</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>1. Submit a new booking request for Product Expo from 10:59 to 13:00 on Orchid Hall.
-2. Read the response and the venue's booking rows.</t>
+          <t>1. Sign in as Venue Staff
+ 2. Open the pending request for 10:59–13:00
+ 3. Attempt to approve it</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>Existing claim: 09:00-11:00. Attempted request: 10:59-13:00. Advertised overlap: 1 minute. Both buffers: 0.</t>
+          <t>Existing: 09:00–11:00 · Requested: 10:59–13:00 · Overlap: 1 minute</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>The new request is refused at submission and no overlapping Pending fixture is inserted. The Coordinator is told that the requested buffered window is unavailable, without disclosure of another event's title or private booking details. Charity Run's prior claim remains unchanged.</t>
+          <t>Approval is blocked and the conflicting 09:00–11:00 booking is identified. The venue never holds two confirmed bookings over the same period</t>
         </is>
       </c>
     </row>
@@ -11303,7 +11307,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 4 (Approval rechecks current buffered availability; T-100)</t>
+          <t>E06-S06 — Scenario 4 (Buffered windows are what must not overlap)</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -11318,30 +11322,28 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>Verify buffer-growth conflicts block approvals until an explicit resolution</t>
+          <t>Verify that two approvals whose advertised times do not overlap but whose buffered windows do should let at most one succeed when processed at the same moment</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>Orchid Hall has setup and turnaround set to 0. Two Pending requests, Charity Run 10:00-12:00 and Alumni Dinner 12:00-14:00, were successfully accepted while their advertised windows were adjacent. Venue Staff then changes setup to 30 minutes and turnaround to 45 minutes.</t>
+          <t>Venue "Riverside Hall" has Setup time 30 and Turnaround time 45; two Pending requests exist on it for 15/01/2027: "Charity Run" 10:00-12:00 and "Alumni Dinner" 12:30-14:00; two Venue Staff accounts are signed in; TEST_DATABASE_URL points at the disposable test schema</t>
         </is>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
-          <t>1. Confirm the buffer edit saves and both Pending rows remain; earlier Charity Run is unflagged and later Alumni Dinner has `buffer_conflict` true under the existing equal-status ordering.
-2. Attempt approval of each request while the buffered conflict remains.
-3. Resolve the conflict using one of these paths: (primary) Venue Staff reject one conflicting Pending request with a reason; (alternative) an authorized Coordinator withdraws/replans one request to a nonconflicting period and resubmits it as needed.
-4. Approve the remaining now-free Pending request. For the alternative path, also approve the replanned request only if it is Pending and conflict-free.</t>
+          <t>1. Trigger approval of both requests concurrently (integration test issues both approvals in parallel transactions)
+  2. Read back both bookings and the venue calendar</t>
         </is>
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>Initially both buffers are 0. After the edit, Charity Run occupies 09:30-12:45 and Alumni Dinner occupies 11:30-14:45; these windows overlap from 11:30 to 12:45.</t>
+          <t>Charity Run buffered: 09:30-12:45 | Alumni Dinner buffered: 12:00-14:45 (advertised times do not overlap; buffered windows overlap 12:00-12:45)</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>Both approvals are refused while the conflict remains, and there is no automatic winner. Equal-status ordering leaves earlier Charity Run unflagged and sets `buffer_conflict` true on later Alumni Dinner. The primary resolution is for Venue Staff to reject one conflicting Pending request with a reason; that row becomes terminal Rejected, and the remaining still-Pending request can then be approved. Alternatively, an authorized Coordinator may withdraw/replan one request to a nonconflicting period; the remaining now-free Pending request and any valid replanned Pending request can then be approved. A Rejected row is never approved.</t>
+          <t>Exactly one booking is Confirmed; the other approval fails with the conflict identified and its request remains Pending; the database exclusion constraint rejected the second write on the buffered range (ADR-003), so TC_E06S06_04 (adjacent, must not conflict) and TC_E06S06_05 (one minute of overlap) continue to hold on buffered windows</t>
         </is>
       </c>
     </row>
@@ -11356,7 +11358,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>E06-S06 - Scenario 5 (Conflicts are per venue, not per event; T-100)</t>
+          <t>E06-S06 — Scenario 5 (Conflicts are per venue, not per event)</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -11371,29 +11373,29 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>Verify one event may confirm overlapping bookings at different venues</t>
+          <t>Verify that approving two requests from the same event on two different venues over the same period should confirm both</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>Event Tech Summit has accepted Pending requests on Seminar Room A and Seminar Room B for 15/01/2027 14:00-16:00 (TC_E06S03_07). Each venue has no conflicting active booking.</t>
+          <t>Event "Tech Summit" has Pending requests on "Seminar Room A" and "Seminar Room B" for 15/01/2027 14:00-16:00 (TC_E06S03_07); venue_staff_1@connectsphere.com is signed in</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
-          <t>1. Approve the Seminar Room A request.
-2. Approve the Seminar Room B request.
-3. Read both venue calendars.</t>
+          <t>1. Approve the "Seminar Room A" request
+  2. Approve the "Seminar Room B" request
+  3. Open the availability calendar for both venues on 15/01/2027</t>
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>Same event and period; different venues.</t>
+          <t>Same event, same period, two venues</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>Both requests are accepted and become Confirmed. Each venue calendar shows its own booking; neither venue's availability check blocks the other. E06-S03's multiple-venue semantics remain unchanged.</t>
+          <t>Both bookings become Confirmed; neither approval is blocked; each venue's calendar shows its own Confirmed period; TC_E06S06_01 to TC_E06S06_06 (conflicts on one venue) continue to hold</t>
         </is>
       </c>
     </row>
@@ -15347,7 +15349,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>E09-S02 - Scenario 5 (Waiting list remains event-level; T-98)</t>
+          <t>E09-S02 - Scenario 5 (Waiting list remains event-level; assumes O-50)</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -15555,7 +15557,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>E09-S02 - Scenario 2 (Over-capacity submission remains Pending); T-98</t>
+          <t>E09-S02 - Scenario 2 (Over-capacity submission remains Pending); assumes O-50</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -15591,7 +15593,7 @@
       </c>
       <c r="J289" s="2" t="inlineStr">
         <is>
-          <t>The request is saved as Pending for Organiser review; it does not consume an approved seat or create a Session waitlist (T-98)</t>
+          <t>The request is saved as Pending for Organiser review; it does not consume an approved seat or create a Session waitlist (assumes O-50)</t>
         </is>
       </c>
     </row>
@@ -16226,7 +16228,7 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>E09-S04 - Scenario 1 (Joined a full Event's list); T-98</t>
+          <t>E09-S04 - Scenario 1 (Joined a full Event's list); assumes O-50</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
@@ -16263,7 +16265,7 @@
       </c>
       <c r="J302" s="2" t="inlineStr">
         <is>
-          <t>attendee_i@example.com is added to the Event-level waiting list and receives confirmation; no Session-specific waiting-list entry is created (T-98)</t>
+          <t>attendee_i@example.com is added to the Event-level waiting list and receives confirmation; no Session-specific waiting-list entry is created (assumes O-50)</t>
         </is>
       </c>
     </row>

</xml_diff>